<commit_message>
Seite-Feld entfernen, automatische Seitenzahl in laufender Kopfzeile
- "Seite" als manuelles Feld aus Vorlage/Beispiel/Parser entfernt
- PDF erhaelt auf JEDER Seite eine laufende Kopfzeile (echte Seitenzahl +
  Name + Schuljahr + Logo), gezeichnet via jsPDF nach dem Rendern
- Bildschirm-Kopfzeile (Klasse no-pdf) ohne Seitenangabe; im PDF ausgeblendet
- groesserer oberer Rand fuer die Kopfzeile; Logo einmalig als dataURL geladen
- Generatoren und README angepasst

Verifiziert: 7-seitiges PDF, "Seite 1".."Seite 7" je einmal im Datenstrom.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/beispiel-zeugnis.xlsx
+++ b/beispiel-zeugnis.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -467,110 +467,114 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Seite</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>3</v>
+          <t>Kommentar</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Du hast an der Theater-AG und an der … AG teilgenommen.
+Lieber Jannes, wir freuen uns auf das vierte Schuljahr mit dir und wünschen dir weiterhin viel Erfolg und Freude beim Lernen!</t>
+        </is>
       </c>
       <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Kommentar</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Du hast an der Theater-AG und an der … AG teilgenommen.
-Lieber Jannes, wir freuen uns auf das vierte Schuljahr mit dir und wünschen dir weiterhin viel Erfolg und Freude beim Lernen!</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
       <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Fach</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Kompetenz</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Subkompetenz</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Bewertung</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Fachkommentar</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Fach</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Kompetenz</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>Subkompetenz</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Bewertung</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>Fachkommentar</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Sprechen und Zuhören</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Du gibst Informationen korrekt wieder.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Jannes beteiligt sich rege am Unterrichtsgespräch.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Deutsch</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Sprechen und Zuhören</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Du gibst Informationen korrekt wieder.</t>
+          <t>Du beziehst dich auf die Beiträge anderer.</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Jannes beteiligt sich rege am Unterrichtsgespräch.</t>
-        </is>
-      </c>
+      <c r="E7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr"/>
       <c r="B8" s="2" t="inlineStr"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Du beziehst dich auf die Beiträge anderer.</t>
+          <t>Du trägst Texte verständlich vor.</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Lesen</t>
+        </is>
+      </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Du trägst Texte verständlich vor.</t>
+          <t>Du liest altersgemäße Texte flüssig, sinnbetont und in angemessenem Tempo, auch wenn der Text dir noch unbekannt ist und längere Sätze enthält.</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
@@ -580,117 +584,100 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Lesen</t>
-        </is>
-      </c>
+      <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Du liest altersgemäße Texte flüssig, sinnbetont und in angemessenem Tempo, auch wenn der Text dir noch unbekannt ist und längere Sätze enthält.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>2</v>
+          <t>Du entnimmst Texten gezielt Informationen.
+Dazu nutzt du Überschriften, Bilder und den Zusammenhang.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Schreiben</t>
+        </is>
+      </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Du entnimmst Texten gezielt Informationen.
-Dazu nutzt du Überschriften, Bilder und den Zusammenhang.</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
+          <t>Du schreibst gut lesbar und formklar.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Schreiben</t>
-        </is>
-      </c>
+      <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Du schreibst gut lesbar und formklar.</t>
+          <t>Du wendest Rechtschreibregeln an.</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="2" t="inlineStr"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Mathematik</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Zahlen und Operationen</t>
+        </is>
+      </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Du wendest Rechtschreibregeln an.</t>
+          <t>Du rechnest im Zahlenraum bis 1000 sicher.</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Mathematik</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Zahlen und Operationen</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Du rechnest im Zahlenraum bis 1000 sicher.</t>
+          <t>Du löst Sachaufgaben selbstständig.</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Größen und Messen</t>
+        </is>
+      </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Du löst Sachaufgaben selbstständig.</t>
+          <t>Du schätzt und misst Längen sachgerecht.</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Größen und Messen</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Du schätzt und misst Längen sachgerecht.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fachkommentar als kursive Zeile unter dem Fach; Vorschau-Kopfzeile
- Fachkommentar ist keine Spalte mehr, sondern eine eigene Zeile unter der
  untersten Kompetenz (Marker "Kommentar" in der Kompetenz-Spalte, Text in der
  Faehigkeit-Spalte); im Zeugnis kursiv und in der Excel-Vorlage kursiv
- Parser/Render/Validierung und beide .xlsx + README entsprechend angepasst
- Vorschau-Kopfzeile: Logo rechts (float), Schuljahr direkt nach dem Namen,
  "Seite 1" wird angezeigt

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/beispiel-zeugnis.xlsx
+++ b/beispiel-zeugnis.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +28,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -50,12 +53,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -424,14 +430,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,7 +452,6 @@
       </c>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -462,7 +466,6 @@
       </c>
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -478,14 +481,12 @@
       </c>
       <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n"/>
       <c r="B4" s="2" t="n"/>
       <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -508,11 +509,6 @@
           <t>Bewertung</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Fachkommentar</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -532,11 +528,6 @@
       </c>
       <c r="D6" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Jannes beteiligt sich rege am Unterrichtsgespräch.</t>
-        </is>
       </c>
     </row>
     <row r="7">
@@ -550,7 +541,6 @@
       <c r="D7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr"/>
@@ -563,7 +553,6 @@
       <c r="D8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr"/>
@@ -580,7 +569,6 @@
       <c r="D9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr"/>
@@ -596,7 +584,6 @@
           <t>*</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr"/>
@@ -613,7 +600,6 @@
       <c r="D11" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr"/>
@@ -626,58 +612,68 @@
       <c r="D12" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Kommentar</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Jannes beteiligt sich rege am Unterrichtsgespräch.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Mathematik</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Zahlen und Operationen</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Du rechnest im Zahlenraum bis 1000 sicher.</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-      <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Du löst Sachaufgaben selbstständig.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Du löst Sachaufgaben selbstständig.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Größen und Messen</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Du schätzt und misst Längen sachgerecht.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D16" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -698,12 +694,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Bewertung</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Bedeutung</t>
         </is>

</xml_diff>